<commit_message>
Segundo commit del proyecto
</commit_message>
<xml_diff>
--- a/dist/incidentes_mes.xlsx
+++ b/dist/incidentes_mes.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LuisAlvaroRojasRinco\Desktop\AutInforme-py\dist\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E393D28-2979-43FD-A4CA-9D48E8E4CB86}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{285B5E45-5044-4485-955F-1D4542850398}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="7890" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="7890" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Incidentes" sheetId="1" r:id="rId1"/>
+    <sheet name="Novedades" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="21">
   <si>
     <t>Codigo</t>
   </si>
@@ -58,7 +59,36 @@
     <t>CRU7032</t>
   </si>
   <si>
-    <t>Rasomware</t>
+    <t>TICKET: INC-16762.
+EVENTO: Falla en la Geolocalización operador Movistar.
+OBSERVACIONES: Se evidencia que no se esta recibiendo datos de geolocalización del Operador Movistar, los demás
+operadores se encuentran con normalidad</t>
+  </si>
+  <si>
+    <t>TICKET:INC-16290.
+EVENTO: Falla en la Geolocalización operador TIGO.
+OBSERVACIONES: Se evidencia que no se esta recibiendo datos de geolocalización del Operador TIGO, los demás operadores se encuentran con normalidad</t>
+  </si>
+  <si>
+    <t>Fecha</t>
+  </si>
+  <si>
+    <t>Novedades</t>
+  </si>
+  <si>
+    <t>Estado</t>
+  </si>
+  <si>
+    <t>ACTIVA</t>
+  </si>
+  <si>
+    <t>CERRADA</t>
+  </si>
+  <si>
+    <t>Ransomware</t>
+  </si>
+  <si>
+    <t>CRU7003</t>
   </si>
 </sst>
 </file>
@@ -94,8 +124,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -398,10 +438,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -467,7 +507,7 @@
         <v>10</v>
       </c>
       <c r="C6" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -478,10 +518,135 @@
         <v>10</v>
       </c>
       <c r="C7" t="s">
-        <v>12</v>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28819674-DB58-40C7-A1F4-2E58262327E5}">
+  <dimension ref="A1:E1048576"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="56.28515625" customWidth="1"/>
+    <col min="4" max="4" width="13.28515625" customWidth="1"/>
+    <col min="5" max="5" width="55.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="75" x14ac:dyDescent="0.25">
+      <c r="C2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="75" x14ac:dyDescent="0.25">
+      <c r="C3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" s="3"/>
+    </row>
+    <row r="4" spans="1:5" ht="75" x14ac:dyDescent="0.25">
+      <c r="C4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="75" x14ac:dyDescent="0.25">
+      <c r="C5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="75" x14ac:dyDescent="0.25">
+      <c r="C6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="75" x14ac:dyDescent="0.25">
+      <c r="C7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="75" x14ac:dyDescent="0.25">
+      <c r="C8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="75" x14ac:dyDescent="0.25">
+      <c r="C9" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C10" s="4"/>
+      <c r="D10" s="2"/>
+    </row>
+    <row r="1048575" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1048575" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="1048576" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1048576" t="s">
+        <v>18</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D10" xr:uid="{1DC309E1-3454-4DE9-BC82-3EDC5FAD46CB}">
+      <formula1>$A$1048575:$A$1048576</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Mejoras UI: Mejora al traer nombres de responsables y Mejora en interfaz
</commit_message>
<xml_diff>
--- a/dist/incidentes_mes.xlsx
+++ b/dist/incidentes_mes.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LuisAlvaroRojasRinco\Desktop\AutInforme-py\dist\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LuisAlvaroRojasRinco\Desktop\Luis-R\Autom\AutInforme-py\dist\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{285B5E45-5044-4485-955F-1D4542850398}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2BA1593-2A8C-42ED-A7B2-A1EAB26D6FD4}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="7890" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="7890" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Incidentes" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="22">
   <si>
     <t>Codigo</t>
   </si>
@@ -89,6 +89,12 @@
   </si>
   <si>
     <t>CRU7003</t>
+  </si>
+  <si>
+    <t>TICKET: INC-16701.
+EVENTO: Falla en la Geolocalización operador TIGO.
+OBSERVACIONES: Se evidencia que no se esta recibiendo datos de geolocalización del Operador TIGO, los demás operadores
+se encuentran con normalidad</t>
   </si>
 </sst>
 </file>
@@ -438,13 +444,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:XFC8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="12.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3 16381:16383" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -455,85 +461,86 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" spans="1:3 16381:16383" x14ac:dyDescent="0.25">
+      <c r="XFA2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="XFB2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" t="s">
+      <c r="XFC2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="3" spans="1:3 16381:16383" x14ac:dyDescent="0.25">
+      <c r="XFA3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" t="s">
+      <c r="XFB3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" t="s">
+      <c r="XFC3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="4" spans="1:3 16381:16383" x14ac:dyDescent="0.25">
+      <c r="XFA4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
+      <c r="XFB4" t="s">
         <v>8</v>
       </c>
-      <c r="C4" t="s">
+      <c r="XFC4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="5" spans="1:3 16381:16383" x14ac:dyDescent="0.25">
+      <c r="XFA5" t="s">
         <v>5</v>
       </c>
-      <c r="B5" t="s">
+      <c r="XFB5" t="s">
         <v>9</v>
       </c>
-      <c r="C5" t="s">
+      <c r="XFC5" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="6" spans="1:3 16381:16383" x14ac:dyDescent="0.25">
+      <c r="XFA6" t="s">
         <v>6</v>
       </c>
-      <c r="B6" t="s">
+      <c r="XFB6" t="s">
         <v>10</v>
       </c>
-      <c r="C6" t="s">
+      <c r="XFC6" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="7" spans="1:3 16381:16383" x14ac:dyDescent="0.25">
+      <c r="XFA7" t="s">
         <v>11</v>
       </c>
-      <c r="B7" t="s">
+      <c r="XFB7" t="s">
         <v>10</v>
       </c>
-      <c r="C7" t="s">
+      <c r="XFC7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="8" spans="1:3 16381:16383" x14ac:dyDescent="0.25">
+      <c r="XFA8" t="s">
         <v>20</v>
       </c>
-      <c r="B8" t="s">
+      <c r="XFB8" t="s">
         <v>10</v>
       </c>
-      <c r="C8" t="s">
+      <c r="XFC8" t="s">
         <v>19</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -566,7 +573,7 @@
         <v>13</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="75" x14ac:dyDescent="0.25">
@@ -574,57 +581,37 @@
         <v>12</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E3" s="3"/>
     </row>
-    <row r="4" spans="1:5" ht="75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" ht="90" x14ac:dyDescent="0.25">
       <c r="C4" s="1" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="75" x14ac:dyDescent="0.25">
-      <c r="C5" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="75" x14ac:dyDescent="0.25">
-      <c r="C6" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="75" x14ac:dyDescent="0.25">
-      <c r="C7" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="75" x14ac:dyDescent="0.25">
-      <c r="C8" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="75" x14ac:dyDescent="0.25">
-      <c r="C9" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>17</v>
-      </c>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C5" s="1"/>
+      <c r="D5" s="2"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C6" s="1"/>
+      <c r="D6" s="2"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C7" s="1"/>
+      <c r="D7" s="2"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C8" s="1"/>
+      <c r="D8" s="2"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C9" s="1"/>
+      <c r="D9" s="2"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C10" s="4"/>

</xml_diff>